<commit_message>
Fix bug and add scenario, update card to close bucket
</commit_message>
<xml_diff>
--- a/testdata/LeadManagement.xlsx
+++ b/testdata/LeadManagement.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Sales Force\Automation\stp-automation-test\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CF4EB7F-B150-4EDC-8FD1-5D3FBDD2A0E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5776B4A4-CDA6-48CF-A78B-90008F7B419D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C7681F3F-D0BE-43DE-AC81-0EAE175E5E0E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{C7681F3F-D0BE-43DE-AC81-0EAE175E5E0E}"/>
   </bookViews>
   <sheets>
     <sheet name="addLeadManagement" sheetId="5" r:id="rId1"/>
     <sheet name="editLeadManagement" sheetId="6" r:id="rId2"/>
     <sheet name="addCallScheduller" sheetId="7" r:id="rId3"/>
+    <sheet name="EditProgressCardBySales" sheetId="9" r:id="rId4"/>
+    <sheet name="editMoveCardToClose" sheetId="8" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="57">
   <si>
     <t>customer</t>
   </si>
@@ -195,6 +197,18 @@
   </si>
   <si>
     <t>Negotation</t>
+  </si>
+  <si>
+    <t>Closing</t>
+  </si>
+  <si>
+    <t>I'll close this card, thank you sir</t>
+  </si>
+  <si>
+    <t>Boss, this card has been deal, thank you</t>
+  </si>
+  <si>
+    <t>Deal</t>
   </si>
 </sst>
 </file>
@@ -829,9 +843,6 @@
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
@@ -969,4 +980,194 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE6C99D6-2A29-4EB1-9BEF-7656C518F079}">
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M1" t="s">
+        <v>29</v>
+      </c>
+      <c r="N1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="N2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="H3" t="s">
+        <v>56</v>
+      </c>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="N3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFDC0414-8A31-48F3-B127-9C153A0B8A75}">
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M1" t="s">
+        <v>29</v>
+      </c>
+      <c r="N1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="N2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="N3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix bug mobile test automation
</commit_message>
<xml_diff>
--- a/testdata/LeadManagement.xlsx
+++ b/testdata/LeadManagement.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Sales Force\Automation\stp-automation-test\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Sales Force\Automation\sales-force-automation-test\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5776B4A4-CDA6-48CF-A78B-90008F7B419D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0D0278-A471-4631-8E03-AE3D60317393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{C7681F3F-D0BE-43DE-AC81-0EAE175E5E0E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{C7681F3F-D0BE-43DE-AC81-0EAE175E5E0E}"/>
   </bookViews>
   <sheets>
     <sheet name="addLeadManagement" sheetId="5" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="51">
   <si>
     <t>customer</t>
   </si>
@@ -148,18 +148,9 @@
     <t>1</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>Cabang Green Garden</t>
-  </si>
-  <si>
     <t>Selling</t>
   </si>
   <si>
-    <t>Penjualan product dari cabang outlet green garden</t>
-  </si>
-  <si>
     <t>3</t>
   </si>
   <si>
@@ -170,15 +161,6 @@
   </si>
   <si>
     <t>Penjualan product dari cabang outlet permata hijau</t>
-  </si>
-  <si>
-    <t>Cabang Permata Hijau</t>
-  </si>
-  <si>
-    <t>Buying</t>
-  </si>
-  <si>
-    <t>Penjualan product dari cabang outlet Kebayoran Lama</t>
   </si>
   <si>
     <t>startTime</t>
@@ -803,7 +785,7 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
@@ -866,7 +848,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5959604A-744E-4A76-8572-7C6F5D39EFF7}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="20.88671875" bestFit="1" customWidth="1"/>
@@ -877,19 +859,19 @@
         <v>7</v>
       </c>
       <c r="B1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D1" t="s">
         <v>0</v>
       </c>
       <c r="E1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="F1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
@@ -906,74 +888,22 @@
         <v>35</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" t="s">
         <v>36</v>
       </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F2" t="s">
-        <v>38</v>
-      </c>
       <c r="G2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3" t="s">
-        <v>38</v>
-      </c>
-      <c r="G3" t="s">
-        <v>43</v>
-      </c>
-      <c r="H3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F4" t="s">
         <v>45</v>
-      </c>
-      <c r="G4" t="s">
-        <v>46</v>
-      </c>
-      <c r="H4" t="s">
-        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1050,7 +980,7 @@
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="N2" t="s">
         <v>30</v>
@@ -1063,7 +993,7 @@
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="H3" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -1145,7 +1075,7 @@
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="N2" t="s">
         <v>30</v>
@@ -1153,7 +1083,7 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>

</xml_diff>